<commit_message>
various fixes after configuring haier study
</commit_message>
<xml_diff>
--- a/output/cumulative-benefit-forecast.xlsx
+++ b/output/cumulative-benefit-forecast.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ecalia-my.sharepoint.com/personal/michael_ilewicz_ecalia_de/Documents/Documents/GitHub/heatpump-calculations/output/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_C2BE00265031921FD2FE31D2F8F2D3C244D21492" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03EC5CBF-8970-49FE-A342-A7E9C8E7A078}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -46,8 +52,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,13 +116,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -154,7 +168,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -188,6 +202,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -222,9 +237,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -397,11 +413,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" customWidth="1"/>
+    <col min="2" max="3" width="16.109375" customWidth="1"/>
+    <col min="4" max="4" width="47.77734375" customWidth="1"/>
+    <col min="5" max="5" width="38.88671875" customWidth="1"/>
+    <col min="6" max="6" width="31.21875" customWidth="1"/>
+    <col min="7" max="7" width="23.88671875" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" customWidth="1"/>
+    <col min="9" max="9" width="22.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -430,7 +456,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -441,25 +467,25 @@
         <v>2658</v>
       </c>
       <c r="D2">
-        <v>20668965.35214449</v>
+        <v>20668965.352144491</v>
       </c>
       <c r="E2">
-        <v>7795149.986770763</v>
+        <v>7795149.9867707631</v>
       </c>
       <c r="F2">
         <v>16274461.58444082</v>
       </c>
       <c r="G2">
-        <v>6137524.82032264</v>
+        <v>6137524.8203226402</v>
       </c>
       <c r="H2">
-        <v>4.394503767703672</v>
+        <v>4.3945037677036716</v>
       </c>
       <c r="I2">
-        <v>1657.625166448123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>1657.6251664481231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2027</v>
       </c>
@@ -470,25 +496,25 @@
         <v>9378</v>
       </c>
       <c r="D3">
-        <v>93591677.30253661</v>
+        <v>93591677.302536607</v>
       </c>
       <c r="E3">
-        <v>35297420.36595096</v>
+        <v>35297420.365950957</v>
       </c>
       <c r="F3">
-        <v>73692653.30384628</v>
+        <v>73692653.303846285</v>
       </c>
       <c r="G3">
-        <v>27791425.47611934</v>
+        <v>27791425.476119339</v>
       </c>
       <c r="H3">
-        <v>19.89902399869032</v>
+        <v>19.899023998690321</v>
       </c>
       <c r="I3">
-        <v>7505.994889831616</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>7505.9948898316161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2028</v>
       </c>
@@ -502,22 +528,22 @@
         <v>209057701.2331264</v>
       </c>
       <c r="E4">
-        <v>78844591.50917406</v>
+        <v>78844591.509174064</v>
       </c>
       <c r="F4">
-        <v>164608875.7361369</v>
+        <v>164608875.73613691</v>
       </c>
       <c r="G4">
-        <v>62078309.04014239</v>
+        <v>62078309.040142387</v>
       </c>
       <c r="H4">
-        <v>44.44882549698947</v>
+        <v>44.448825496989471</v>
       </c>
       <c r="I4">
         <v>16766.28246903167</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2029</v>
       </c>
@@ -528,25 +554,25 @@
         <v>15848</v>
       </c>
       <c r="D5">
-        <v>446552669.8219881</v>
+        <v>446552669.82198811</v>
       </c>
       <c r="E5">
         <v>168414091.6129224</v>
       </c>
       <c r="F5">
-        <v>351608863.4360959</v>
+        <v>351608863.43609589</v>
       </c>
       <c r="G5">
         <v>132600891.6217684</v>
       </c>
       <c r="H5">
-        <v>94.9438063858922</v>
+        <v>94.943806385892202</v>
       </c>
       <c r="I5">
-        <v>35813.19999115396</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <v>35813.199991153961</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2030</v>
       </c>
@@ -557,25 +583,25 @@
         <v>20603</v>
       </c>
       <c r="D6">
-        <v>930079456.6385953</v>
+        <v>930079456.63859534</v>
       </c>
       <c r="E6">
-        <v>350772702.4632108</v>
+        <v>350772702.46321082</v>
       </c>
       <c r="F6">
-        <v>732330524.8002999</v>
+        <v>732330524.80029988</v>
       </c>
       <c r="G6">
-        <v>276180980.1357231</v>
+        <v>276180980.13572311</v>
       </c>
       <c r="H6">
         <v>197.7489318382955</v>
       </c>
       <c r="I6">
-        <v>74591.72232748767</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>74591.722327487674</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2031</v>
       </c>
@@ -586,25 +612,25 @@
         <v>26783</v>
       </c>
       <c r="D7">
-        <v>1908215182.829826</v>
+        <v>1908215182.8298261</v>
       </c>
       <c r="E7">
-        <v>719669477.5218443</v>
+        <v>719669477.52184427</v>
       </c>
       <c r="F7">
-        <v>1502499880.929691</v>
+        <v>1502499880.9296911</v>
       </c>
       <c r="G7">
-        <v>566631972.5195096</v>
+        <v>566631972.51950955</v>
       </c>
       <c r="H7">
         <v>405.7153019001347</v>
       </c>
       <c r="I7">
-        <v>153037.5050023347</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>153037.50500233471</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2032</v>
       </c>
@@ -615,25 +641,25 @@
         <v>34818</v>
       </c>
       <c r="D8">
-        <v>3878910871.258421</v>
+        <v>3878910871.2584209</v>
       </c>
       <c r="E8">
         <v>1462903023.332294</v>
       </c>
       <c r="F8">
-        <v>3054195998.591051</v>
+        <v>3054195998.5910511</v>
       </c>
       <c r="G8">
-        <v>1151817131.66737</v>
+        <v>1151817131.6673701</v>
       </c>
       <c r="H8">
-        <v>824.714872667371</v>
+        <v>824.71487266737097</v>
       </c>
       <c r="I8">
-        <v>311085.8916649239</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>311085.89166492393</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2033</v>
       </c>
@@ -650,7 +676,7 @@
         <v>2956440229.516367</v>
       </c>
       <c r="F9">
-        <v>6172348844.396247</v>
+        <v>6172348844.3962469</v>
       </c>
       <c r="G9">
         <v>2327754061.827373</v>
@@ -659,10 +685,10 @@
         <v>1666.699926422717</v>
       </c>
       <c r="I9">
-        <v>628686.1676889943</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>628686.16768899432</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2034</v>
       </c>
@@ -676,22 +702,22 @@
         <v>15783695337.25444</v>
       </c>
       <c r="E10">
-        <v>5952705899.59631</v>
+        <v>5952705899.5963097</v>
       </c>
       <c r="F10">
-        <v>12427843776.40706</v>
+        <v>12427843776.407061</v>
       </c>
       <c r="G10">
-        <v>4686864686.270123</v>
+        <v>4686864686.2701225</v>
       </c>
       <c r="H10">
-        <v>3355.851560847377</v>
+        <v>3355.8515608473772</v>
       </c>
       <c r="I10">
-        <v>1265841.213326187</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>1265841.2133261871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2035</v>
       </c>
@@ -702,25 +728,25 @@
         <v>76496</v>
       </c>
       <c r="D11">
-        <v>31704653929.90103</v>
+        <v>31704653929.901031</v>
       </c>
       <c r="E11">
-        <v>11957179637.7475</v>
+        <v>11957179637.747499</v>
       </c>
       <c r="F11">
-        <v>24963766679.23015</v>
+        <v>24963766679.230148</v>
       </c>
       <c r="G11">
-        <v>9414488835.832144</v>
+        <v>9414488835.8321438</v>
       </c>
       <c r="H11">
-        <v>6740.887250670885</v>
+        <v>6740.8872506708849</v>
       </c>
       <c r="I11">
-        <v>2542690.801915358</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>2542690.8019153578</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2036</v>
       </c>
@@ -731,22 +757,22 @@
         <v>99445</v>
       </c>
       <c r="D12">
-        <v>63587758607.38281</v>
+        <v>63587758607.382813</v>
       </c>
       <c r="E12">
-        <v>23981660676.9867</v>
+        <v>23981660676.986698</v>
       </c>
       <c r="F12">
-        <v>50068042728.6534</v>
+        <v>50068042728.653397</v>
       </c>
       <c r="G12">
         <v>18881967427.2813</v>
       </c>
       <c r="H12">
-        <v>13519.71587872942</v>
+        <v>13519.715878729419</v>
       </c>
       <c r="I12">
-        <v>5099693.249705401</v>
+        <v>5099693.2497054012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>